<commit_message>
Source annotations v2: connectivity + verified paid gating only
Per feedback, drop implementation-centric labels (待开发插件/需API密钥)
from all source annotations and docs; the taxonomy is now purely
source-centric: 联通·可取数 / 联通·暂无数据 / 联通·免费 / 联通·需付费
(verified) / 不可联通 / 无链接未验证. The 需付费 label is backed by a
real HTTP probe of each vendor endpoint (404 URLs probed via proxy,
status codes recorded — 401/403 corroborate gating) cross-checked with
the workbook's 是否付费 column. Regenerated: annotated workbook +
per-sheet splits + connectivity_report.csv (adds 是否付费/联通状态/
联通说明/url_probe columns); rewrote SOURCES_CONNECTIVITY.zh-CN.md and
the API-reference landscape sections (EN+zh) to the new taxonomy.

Result over 1232 sources: 931 reachable (491 serving data, 310 paid,
64 free official APIs, 66 empty), 240 unreachable, 61 no URL.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reports/连通标注_2026-07-04_分表/1_新闻.xlsx
+++ b/docs/reports/连通标注_2026-07-04_分表/1_新闻.xlsx
@@ -1461,7 +1461,7 @@
       </c>
       <c r="K3" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K4" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K5" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="K6" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="K7" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="K8" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="K9" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="K10" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="K11" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="K12" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="K13" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="K14" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="K15" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="K16" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="K17" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="K18" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="K19" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="K20" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="K21" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="K22" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="K23" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="K24" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="K25" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="K26" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="K27" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="K28" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="K29" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="K30" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="K31" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="K32" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="K33" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="K34" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="K35" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="K36" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="K37" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -3520,7 +3520,7 @@
       </c>
       <c r="K38" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="K39" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="K40" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="K41" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="K42" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="K43" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="K44" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="K45" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3985,12 +3985,12 @@
       </c>
       <c r="K46" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4045,7 @@
       </c>
       <c r="K47" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="K48" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="K49" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="K50" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="K51" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="K52" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="K53" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="K54" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="K55" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4567,12 +4567,12 @@
       </c>
       <c r="K56" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K57" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="K58" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="K59" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="K60" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="K61" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="K62" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="K63" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="K64" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="K65" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="K66" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="K67" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="K68" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="K69" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="K70" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="K71" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -5441,12 +5441,12 @@
       </c>
       <c r="K72" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -5495,12 +5495,12 @@
       </c>
       <c r="K73" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -5549,12 +5549,12 @@
       </c>
       <c r="K74" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -5603,12 +5603,12 @@
       </c>
       <c r="K75" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -5657,7 +5657,7 @@
       </c>
       <c r="K76" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="K77" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="K78" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="K79" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="K80" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -5941,7 +5941,7 @@
       </c>
       <c r="K81" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="K82" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="K83" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="K84" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -6169,7 +6169,7 @@
       </c>
       <c r="K85" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -6223,7 +6223,7 @@
       </c>
       <c r="K86" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="K87" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="K88" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="K89" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="K90" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="K91" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="K92" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="K93" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="K94" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="K95" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="K96" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -6829,12 +6829,12 @@
       </c>
       <c r="K97" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="K98" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="K99" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="K100" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="K101" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="K102" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="K103" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="K104" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="K105" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7321,7 +7321,7 @@
       </c>
       <c r="K106" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -7375,7 +7375,7 @@
       </c>
       <c r="K107" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7429,7 +7429,7 @@
       </c>
       <c r="K108" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="K109" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K110" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7597,7 +7597,7 @@
       </c>
       <c r="K111" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="K112" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="K113" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="K114" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7825,7 +7825,7 @@
       </c>
       <c r="K115" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -7879,7 +7879,7 @@
       </c>
       <c r="K116" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="K117" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7991,7 +7991,7 @@
       </c>
       <c r="K118" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -8045,12 +8045,12 @@
       </c>
       <c r="K119" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>HTTP 403,反爬/拒绝访问</t>
+          <t>HTTP 403,访问被拒</t>
         </is>
       </c>
     </row>
@@ -8099,7 +8099,7 @@
       </c>
       <c r="K120" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="K121" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8207,7 +8207,7 @@
       </c>
       <c r="K122" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="K123" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="K124" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8369,7 +8369,7 @@
       </c>
       <c r="K125" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="K126" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8477,7 +8477,7 @@
       </c>
       <c r="K127" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8535,7 +8535,7 @@
       </c>
       <c r="K128" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="K129" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="K130" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="K131" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="K132" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="K133" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="K134" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -8917,7 +8917,7 @@
       </c>
       <c r="K135" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="K136" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -9025,7 +9025,7 @@
       </c>
       <c r="K137" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="K138" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="K139" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -9197,7 +9197,7 @@
       </c>
       <c r="K140" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="K141" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="K142" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="K143" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="K144" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="K145" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -9555,7 +9555,7 @@
       </c>
       <c r="K146" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="K147" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -9673,7 +9673,7 @@
       </c>
       <c r="K148" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="K149" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="K150" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -9847,7 +9847,7 @@
       </c>
       <c r="K151" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="K152" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="K153" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -10024,7 +10024,7 @@
       </c>
       <c r="K154" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -10083,7 +10083,7 @@
       </c>
       <c r="K155" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -10142,7 +10142,7 @@
       </c>
       <c r="K156" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -10201,7 +10201,7 @@
       </c>
       <c r="K157" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -10259,7 +10259,7 @@
       </c>
       <c r="K158" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">
@@ -10317,7 +10317,7 @@
       </c>
       <c r="K159" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
@@ -10375,7 +10375,7 @@
       </c>
       <c r="K160" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
@@ -10433,7 +10433,7 @@
       </c>
       <c r="K161" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L161" t="inlineStr">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="K162" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L162" t="inlineStr">
@@ -10549,7 +10549,7 @@
       </c>
       <c r="K163" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="K164" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="K165" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -10724,7 +10724,7 @@
       </c>
       <c r="K166" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="K167" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
@@ -10840,7 +10840,7 @@
       </c>
       <c r="K168" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
@@ -10898,7 +10898,7 @@
       </c>
       <c r="K169" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="K170" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
@@ -11015,7 +11015,7 @@
       </c>
       <c r="K171" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
@@ -11073,7 +11073,7 @@
       </c>
       <c r="K172" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -11133,7 +11133,7 @@
       </c>
       <c r="K173" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
@@ -11191,7 +11191,7 @@
       </c>
       <c r="K174" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="K175" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="K176" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
@@ -11366,7 +11366,7 @@
       </c>
       <c r="K177" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="K178" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -11482,7 +11482,7 @@
       </c>
       <c r="K179" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
@@ -11540,7 +11540,7 @@
       </c>
       <c r="K180" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
@@ -11598,7 +11598,7 @@
       </c>
       <c r="K181" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="K182" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L182" t="inlineStr">
@@ -11714,12 +11714,12 @@
       </c>
       <c r="K183" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>HTTP 403,反爬/拒绝访问</t>
+          <t>HTTP 403,访问被拒</t>
         </is>
       </c>
     </row>
@@ -11772,7 +11772,7 @@
       </c>
       <c r="K184" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L184" t="inlineStr">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="K185" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L185" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="K186" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L186" t="inlineStr">
@@ -11944,7 +11944,7 @@
       </c>
       <c r="K187" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L187" t="inlineStr">
@@ -12003,7 +12003,7 @@
       </c>
       <c r="K188" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L188" t="inlineStr">
@@ -12062,7 +12062,7 @@
       </c>
       <c r="K189" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L189" t="inlineStr">
@@ -12121,7 +12121,7 @@
       </c>
       <c r="K190" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L190" t="inlineStr">
@@ -12180,7 +12180,7 @@
       </c>
       <c r="K191" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L191" t="inlineStr">
@@ -12239,7 +12239,7 @@
       </c>
       <c r="K192" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L192" t="inlineStr">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="K193" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
@@ -12356,7 +12356,7 @@
       </c>
       <c r="K194" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L194" t="inlineStr">
@@ -12415,7 +12415,7 @@
       </c>
       <c r="K195" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L195" t="inlineStr">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="K196" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L196" t="inlineStr">
@@ -12531,7 +12531,7 @@
       </c>
       <c r="K197" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L197" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="K198" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L198" t="inlineStr">
@@ -12647,7 +12647,7 @@
       </c>
       <c r="K199" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -12705,7 +12705,7 @@
       </c>
       <c r="K200" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L200" t="inlineStr">
@@ -12763,7 +12763,7 @@
       </c>
       <c r="K201" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="K202" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -12879,7 +12879,7 @@
       </c>
       <c r="K203" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
@@ -12937,7 +12937,7 @@
       </c>
       <c r="K204" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L204" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="K205" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L205" t="inlineStr">
@@ -13054,7 +13054,7 @@
       </c>
       <c r="K206" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
@@ -13112,7 +13112,7 @@
       </c>
       <c r="K207" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L207" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="K208" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L208" t="inlineStr">
@@ -13228,7 +13228,7 @@
       </c>
       <c r="K209" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="K210" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L210" t="inlineStr">
@@ -13344,7 +13344,7 @@
       </c>
       <c r="K211" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L211" t="inlineStr">
@@ -13402,7 +13402,7 @@
       </c>
       <c r="K212" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L212" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="K213" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L213" t="inlineStr">
@@ -13519,7 +13519,7 @@
       </c>
       <c r="K214" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L214" t="inlineStr">
@@ -13577,7 +13577,7 @@
       </c>
       <c r="K215" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
@@ -13636,7 +13636,7 @@
       </c>
       <c r="K216" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L216" t="inlineStr">
@@ -13694,7 +13694,7 @@
       </c>
       <c r="K217" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L217" t="inlineStr">
@@ -13752,7 +13752,7 @@
       </c>
       <c r="K218" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L218" t="inlineStr">
@@ -13810,7 +13810,7 @@
       </c>
       <c r="K219" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L219" t="inlineStr">
@@ -13869,7 +13869,7 @@
       </c>
       <c r="K220" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L220" t="inlineStr">
@@ -13928,7 +13928,7 @@
       </c>
       <c r="K221" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L221" t="inlineStr">
@@ -13986,7 +13986,7 @@
       </c>
       <c r="K222" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="K223" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L223" t="inlineStr">
@@ -14098,7 +14098,7 @@
       </c>
       <c r="K224" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L224" t="inlineStr">
@@ -14152,7 +14152,7 @@
       </c>
       <c r="K225" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L225" t="inlineStr">
@@ -14206,7 +14206,7 @@
       </c>
       <c r="K226" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L226" t="inlineStr">
@@ -14264,7 +14264,7 @@
       </c>
       <c r="K227" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L227" t="inlineStr">
@@ -14318,7 +14318,7 @@
       </c>
       <c r="K228" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L228" t="inlineStr">
@@ -14372,7 +14372,7 @@
       </c>
       <c r="K229" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L229" t="inlineStr">
@@ -14426,7 +14426,7 @@
       </c>
       <c r="K230" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L230" t="inlineStr">
@@ -14484,7 +14484,7 @@
       </c>
       <c r="K231" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L231" t="inlineStr">
@@ -14538,7 +14538,7 @@
       </c>
       <c r="K232" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L232" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="K233" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L233" t="inlineStr">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="K234" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L234" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="K235" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L235" t="inlineStr">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="K236" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
@@ -14808,7 +14808,7 @@
       </c>
       <c r="K237" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L237" t="inlineStr">
@@ -14862,7 +14862,7 @@
       </c>
       <c r="K238" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L238" t="inlineStr">
@@ -14916,7 +14916,7 @@
       </c>
       <c r="K239" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L239" t="inlineStr">
@@ -14970,7 +14970,7 @@
       </c>
       <c r="K240" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L240" t="inlineStr">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="K241" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
@@ -15078,7 +15078,7 @@
       </c>
       <c r="K242" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="K243" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L243" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="K244" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
@@ -15240,7 +15240,7 @@
       </c>
       <c r="K245" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
@@ -15294,7 +15294,7 @@
       </c>
       <c r="K246" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L246" t="inlineStr">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="K247" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
@@ -15402,7 +15402,7 @@
       </c>
       <c r="K248" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="K249" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
@@ -15510,7 +15510,7 @@
       </c>
       <c r="K250" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L250" t="inlineStr">
@@ -15564,7 +15564,7 @@
       </c>
       <c r="K251" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L251" t="inlineStr">
@@ -15618,7 +15618,7 @@
       </c>
       <c r="K252" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L252" t="inlineStr">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="K253" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L253" t="inlineStr">
@@ -15726,7 +15726,7 @@
       </c>
       <c r="K254" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L254" t="inlineStr">
@@ -15780,7 +15780,7 @@
       </c>
       <c r="K255" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L255" t="inlineStr">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="K256" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L256" t="inlineStr">
@@ -15888,12 +15888,12 @@
       </c>
       <c r="K257" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -15942,7 +15942,7 @@
       </c>
       <c r="K258" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L258" t="inlineStr">
@@ -15996,7 +15996,7 @@
       </c>
       <c r="K259" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L259" t="inlineStr">
@@ -16050,7 +16050,7 @@
       </c>
       <c r="K260" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L260" t="inlineStr">
@@ -16104,7 +16104,7 @@
       </c>
       <c r="K261" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="K262" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
@@ -16212,7 +16212,7 @@
       </c>
       <c r="K263" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L263" t="inlineStr">
@@ -16266,7 +16266,7 @@
       </c>
       <c r="K264" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L264" t="inlineStr">
@@ -16320,7 +16320,7 @@
       </c>
       <c r="K265" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L265" t="inlineStr">
@@ -16378,7 +16378,7 @@
       </c>
       <c r="K266" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L266" t="inlineStr">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="K267" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L267" t="inlineStr">
@@ -16490,7 +16490,7 @@
       </c>
       <c r="K268" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L268" t="inlineStr">
@@ -16544,7 +16544,7 @@
       </c>
       <c r="K269" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L269" t="inlineStr">
@@ -16598,7 +16598,7 @@
       </c>
       <c r="K270" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L270" t="inlineStr">
@@ -16652,7 +16652,7 @@
       </c>
       <c r="K271" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
@@ -16706,7 +16706,7 @@
       </c>
       <c r="K272" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
@@ -16760,7 +16760,7 @@
       </c>
       <c r="K273" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
@@ -16814,7 +16814,7 @@
       </c>
       <c r="K274" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -16868,7 +16868,7 @@
       </c>
       <c r="K275" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
@@ -16922,7 +16922,7 @@
       </c>
       <c r="K276" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="K277" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="K278" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
@@ -17084,7 +17084,7 @@
       </c>
       <c r="K279" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
@@ -17138,12 +17138,12 @@
       </c>
       <c r="K280" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -17192,7 +17192,7 @@
       </c>
       <c r="K281" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
@@ -17246,12 +17246,12 @@
       </c>
       <c r="K282" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -17300,7 +17300,7 @@
       </c>
       <c r="K283" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
@@ -17354,7 +17354,7 @@
       </c>
       <c r="K284" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
@@ -17408,7 +17408,7 @@
       </c>
       <c r="K285" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
@@ -17462,7 +17462,7 @@
       </c>
       <c r="K286" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L286" t="inlineStr">
@@ -17516,7 +17516,7 @@
       </c>
       <c r="K287" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
@@ -17570,7 +17570,7 @@
       </c>
       <c r="K288" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
@@ -17624,7 +17624,7 @@
       </c>
       <c r="K289" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L289" t="inlineStr">
@@ -17678,7 +17678,7 @@
       </c>
       <c r="K290" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L290" t="inlineStr">
@@ -17732,12 +17732,12 @@
       </c>
       <c r="K291" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -17791,7 +17791,7 @@
       </c>
       <c r="K292" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L292" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="K293" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L293" t="inlineStr">
@@ -17909,7 +17909,7 @@
       </c>
       <c r="K294" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L294" t="inlineStr">
@@ -17968,7 +17968,7 @@
       </c>
       <c r="K295" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L295" t="inlineStr">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="K296" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L296" t="inlineStr">
@@ -18086,7 +18086,7 @@
       </c>
       <c r="K297" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L297" t="inlineStr">
@@ -18144,7 +18144,7 @@
       </c>
       <c r="K298" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
@@ -18203,7 +18203,7 @@
       </c>
       <c r="K299" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
@@ -18261,7 +18261,7 @@
       </c>
       <c r="K300" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L300" t="inlineStr">
@@ -18319,7 +18319,7 @@
       </c>
       <c r="K301" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
@@ -18377,7 +18377,7 @@
       </c>
       <c r="K302" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
@@ -18435,7 +18435,7 @@
       </c>
       <c r="K303" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L303" t="inlineStr">
@@ -18493,7 +18493,7 @@
       </c>
       <c r="K304" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L304" t="inlineStr">
@@ -18551,7 +18551,7 @@
       </c>
       <c r="K305" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L305" t="inlineStr">
@@ -18609,7 +18609,7 @@
       </c>
       <c r="K306" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L306" t="inlineStr">
@@ -18668,7 +18668,7 @@
       </c>
       <c r="K307" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L307" t="inlineStr">
@@ -18726,7 +18726,7 @@
       </c>
       <c r="K308" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L308" t="inlineStr">
@@ -18786,7 +18786,7 @@
       </c>
       <c r="K309" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L309" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="K310" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L310" t="inlineStr">
@@ -18900,7 +18900,7 @@
       </c>
       <c r="K311" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L311" t="inlineStr">
@@ -18954,7 +18954,7 @@
       </c>
       <c r="K312" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L312" t="inlineStr">
@@ -19008,7 +19008,7 @@
       </c>
       <c r="K313" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L313" t="inlineStr">
@@ -19062,7 +19062,7 @@
       </c>
       <c r="K314" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L314" t="inlineStr">
@@ -19116,7 +19116,7 @@
       </c>
       <c r="K315" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L315" t="inlineStr">
@@ -19170,7 +19170,7 @@
       </c>
       <c r="K316" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L316" t="inlineStr">
@@ -19224,7 +19224,7 @@
       </c>
       <c r="K317" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L317" t="inlineStr">
@@ -19278,7 +19278,7 @@
       </c>
       <c r="K318" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L318" t="inlineStr">
@@ -19332,7 +19332,7 @@
       </c>
       <c r="K319" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L319" t="inlineStr">
@@ -19386,7 +19386,7 @@
       </c>
       <c r="K320" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L320" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="K321" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L321" t="inlineStr">
@@ -19494,7 +19494,7 @@
       </c>
       <c r="K322" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L322" t="inlineStr">
@@ -19548,7 +19548,7 @@
       </c>
       <c r="K323" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L323" t="inlineStr">
@@ -19602,7 +19602,7 @@
       </c>
       <c r="K324" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L324" t="inlineStr">
@@ -19656,7 +19656,7 @@
       </c>
       <c r="K325" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L325" t="inlineStr">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="K326" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L326" t="inlineStr">
@@ -19764,7 +19764,7 @@
       </c>
       <c r="K327" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L327" t="inlineStr">
@@ -19818,7 +19818,7 @@
       </c>
       <c r="K328" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L328" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="K329" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L329" t="inlineStr">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="K330" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L330" t="inlineStr">
@@ -19980,7 +19980,7 @@
       </c>
       <c r="K331" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L331" t="inlineStr">
@@ -20034,7 +20034,7 @@
       </c>
       <c r="K332" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L332" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="K333" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L333" t="inlineStr">
@@ -20152,7 +20152,7 @@
       </c>
       <c r="K334" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L334" t="inlineStr">
@@ -20210,7 +20210,7 @@
       </c>
       <c r="K335" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L335" t="inlineStr">
@@ -20268,7 +20268,7 @@
       </c>
       <c r="K336" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L336" t="inlineStr">
@@ -20326,7 +20326,7 @@
       </c>
       <c r="K337" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L337" t="inlineStr">
@@ -20384,7 +20384,7 @@
       </c>
       <c r="K338" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L338" t="inlineStr">
@@ -20442,7 +20442,7 @@
       </c>
       <c r="K339" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L339" t="inlineStr">
@@ -20500,7 +20500,7 @@
       </c>
       <c r="K340" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L340" t="inlineStr">
@@ -20558,7 +20558,7 @@
       </c>
       <c r="K341" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L341" t="inlineStr">
@@ -20616,7 +20616,7 @@
       </c>
       <c r="K342" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L342" t="inlineStr">
@@ -20674,7 +20674,7 @@
       </c>
       <c r="K343" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L343" t="inlineStr">
@@ -20732,7 +20732,7 @@
       </c>
       <c r="K344" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L344" t="inlineStr">
@@ -20790,7 +20790,7 @@
       </c>
       <c r="K345" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L345" t="inlineStr">
@@ -20848,7 +20848,7 @@
       </c>
       <c r="K346" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L346" t="inlineStr">
@@ -20906,7 +20906,7 @@
       </c>
       <c r="K347" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L347" t="inlineStr">
@@ -20964,7 +20964,7 @@
       </c>
       <c r="K348" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L348" t="inlineStr">
@@ -21022,7 +21022,7 @@
       </c>
       <c r="K349" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L349" t="inlineStr">
@@ -21080,7 +21080,7 @@
       </c>
       <c r="K350" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L350" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="K351" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L351" t="inlineStr">
@@ -21196,7 +21196,7 @@
       </c>
       <c r="K352" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L352" t="inlineStr">
@@ -21254,7 +21254,7 @@
       </c>
       <c r="K353" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
@@ -21312,7 +21312,7 @@
       </c>
       <c r="K354" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L354" t="inlineStr">
@@ -21370,7 +21370,7 @@
       </c>
       <c r="K355" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L355" t="inlineStr">
@@ -21428,7 +21428,7 @@
       </c>
       <c r="K356" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
@@ -21486,7 +21486,7 @@
       </c>
       <c r="K357" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
@@ -21544,7 +21544,7 @@
       </c>
       <c r="K358" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L358" t="inlineStr">
@@ -21602,7 +21602,7 @@
       </c>
       <c r="K359" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L359" t="inlineStr">
@@ -21660,7 +21660,7 @@
       </c>
       <c r="K360" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
@@ -21718,7 +21718,7 @@
       </c>
       <c r="K361" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L361" t="inlineStr">
@@ -21776,7 +21776,7 @@
       </c>
       <c r="K362" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L362" t="inlineStr">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="K363" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
@@ -21892,7 +21892,7 @@
       </c>
       <c r="K364" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L364" t="inlineStr">
@@ -21950,7 +21950,7 @@
       </c>
       <c r="K365" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L365" t="inlineStr">
@@ -22008,7 +22008,7 @@
       </c>
       <c r="K366" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L366" t="inlineStr">
@@ -22066,7 +22066,7 @@
       </c>
       <c r="K367" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L367" t="inlineStr">
@@ -22124,7 +22124,7 @@
       </c>
       <c r="K368" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L368" t="inlineStr">
@@ -22182,7 +22182,7 @@
       </c>
       <c r="K369" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L369" t="inlineStr">
@@ -22240,7 +22240,7 @@
       </c>
       <c r="K370" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L370" t="inlineStr">
@@ -22298,12 +22298,12 @@
       </c>
       <c r="K371" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -22356,12 +22356,12 @@
       </c>
       <c r="K372" s="184" t="inlineStr">
         <is>
-          <t>❌ 失败</t>
+          <t>❌ 不可联通</t>
         </is>
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>HTTP 403,反爬/拒绝访问</t>
+          <t>HTTP 403,访问被拒</t>
         </is>
       </c>
     </row>
@@ -22414,7 +22414,7 @@
       </c>
       <c r="K373" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L373" t="inlineStr">
@@ -22468,7 +22468,7 @@
       </c>
       <c r="K374" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L374" t="inlineStr">
@@ -22522,7 +22522,7 @@
       </c>
       <c r="K375" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L375" t="inlineStr">
@@ -22581,12 +22581,12 @@
       </c>
       <c r="K376" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -22640,12 +22640,12 @@
       </c>
       <c r="K377" s="183" t="inlineStr">
         <is>
-          <t>⚠️ 联通但为空</t>
+          <t>⚠️ 联通·暂无数据</t>
         </is>
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>请求成功但解析出 0 条(feed 为空或格式不符)</t>
+          <t>请求成功但当前无内容</t>
         </is>
       </c>
     </row>
@@ -22694,7 +22694,7 @@
       </c>
       <c r="K378" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L378" t="inlineStr">
@@ -22748,7 +22748,7 @@
       </c>
       <c r="K379" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L379" t="inlineStr">
@@ -22802,7 +22802,7 @@
       </c>
       <c r="K380" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L380" t="inlineStr">
@@ -22856,7 +22856,7 @@
       </c>
       <c r="K381" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L381" t="inlineStr">
@@ -22910,7 +22910,7 @@
       </c>
       <c r="K382" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L382" t="inlineStr">
@@ -22964,7 +22964,7 @@
       </c>
       <c r="K383" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L383" t="inlineStr">
@@ -23018,7 +23018,7 @@
       </c>
       <c r="K384" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L384" t="inlineStr">
@@ -23077,7 +23077,7 @@
       </c>
       <c r="K385" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
@@ -23131,7 +23131,7 @@
       </c>
       <c r="K386" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L386" t="inlineStr">
@@ -23185,7 +23185,7 @@
       </c>
       <c r="K387" s="182" t="inlineStr">
         <is>
-          <t>✅ 联通可取数</t>
+          <t>✅ 联通·可取数</t>
         </is>
       </c>
       <c r="L387" t="inlineStr">

</xml_diff>